<commit_message>
Report verified calibration-only alarm refinement failures
</commit_message>
<xml_diff>
--- a/ESA_thesis_results_full_and_historical.xlsx
+++ b/ESA_thesis_results_full_and_historical.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thesis results" sheetId="1" r:id="Rbbb9538c196048fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thesis results" sheetId="1" r:id="R15069f2eeb534f0d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -479,9 +479,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">System-level evaluation. All 2007–2013 entries first, including boundary-sample and planned assessments; other years follow.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">One row per technique. Historical best = highest reported assessment F0.5; descriptive selection, not independent validation.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Technique</x:t>
@@ -1056,8 +1053,8 @@
       <x:c r="L3" s="1"/>
     </x:row>
     <x:row r="4" ht="32" hidden="0" customHeight="1">
-      <x:c r="A4" s="1" t="s">
-        <x:v>2</x:v>
+      <x:c r="A4" s="1" t="str">
+        <x:v>One row per technique. Best reported system F0.5 is descriptive selection, not independent validation.</x:v>
       </x:c>
       <x:c r="B4" s="1"/>
       <x:c r="C4" s="1"/>
@@ -1073,43 +1070,43 @@
     </x:row>
     <x:row r="5" ht="38" hidden="0" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B5" s="3" t="s">
+      <x:c r="C5" s="3" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C5" s="3" t="s">
+      <x:c r="D5" s="3" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D5" s="3" t="s">
+      <x:c r="E5" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E5" s="3" t="s">
+      <x:c r="F5" s="3" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="F5" s="3" t="s">
+      <x:c r="G5" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="G5" s="3" t="s">
+      <x:c r="H5" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="H5" s="3" t="s">
+      <x:c r="I5" s="3" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="I5" s="3" t="s">
+      <x:c r="J5" s="3" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="J5" s="3" t="s">
+      <x:c r="K5" s="3" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="K5" s="3" t="s">
+      <x:c r="L5" s="3" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="L5" s="3" t="s">
+      <x:c r="M5" s="3" t="s">
         <x:v>14</x:v>
-      </x:c>
-      <x:c r="M5" s="3" t="s">
-        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26" hidden="0" customHeight="1">
@@ -1519,7 +1516,7 @@
         <x:v>0.8443148594326733</x:v>
       </x:c>
       <x:c r="M15" s="14" t="str">
-        <x:v>Complete</x:v>
+        <x:v>Original rule retained</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" hidden="0" customHeight="1">
@@ -1560,7 +1557,7 @@
         <x:v>0.8173525522097386</x:v>
       </x:c>
       <x:c r="M16" s="15" t="str">
-        <x:v>Complete. Extra inputs</x:v>
+        <x:v>Original remains best</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="26" hidden="0" customHeight="1">
@@ -2721,9 +2718,9 @@
     <x:row r="70" ht="32" hidden="0" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f9aa8af11be424a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6f4ab9d76a94baf"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re78014510c2c48c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79c235680bbf4456"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify short-no-roll continuation retained original model and results
</commit_message>
<xml_diff>
--- a/ESA_thesis_results_full_and_historical.xlsx
+++ b/ESA_thesis_results_full_and_historical.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thesis results" sheetId="1" r:id="R15069f2eeb534f0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thesis results" sheetId="1" r:id="R0eae2c0a913e4ab5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1188,7 +1188,7 @@
         <x:v>0.907139530369058</x:v>
       </x:c>
       <x:c r="M7" s="1" t="str">
-        <x:v>Complete</x:v>
+        <x:v>Original retained</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26" hidden="0" customHeight="1">
@@ -2718,9 +2718,9 @@
     <x:row r="70" ht="32" hidden="0" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6f4ab9d76a94baf"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53a7f9027438424f"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79c235680bbf4456"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cae9c66e41e45bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify and report nine-run W&B fine-tuning comparison
</commit_message>
<xml_diff>
--- a/ESA_thesis_results_full_and_historical.xlsx
+++ b/ESA_thesis_results_full_and_historical.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thesis results" sheetId="1" r:id="R0eae2c0a913e4ab5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thesis results" sheetId="1" r:id="Rb27b54676ded44e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1054,7 +1054,7 @@
     </x:row>
     <x:row r="4" ht="32" hidden="0" customHeight="1">
       <x:c r="A4" s="1" t="str">
-        <x:v>One row per technique. Best reported system F0.5 is descriptive selection, not independent validation.</x:v>
+        <x:v>One row per technique. The three W&amp;B methods show calibration-selected results; historical bests remain descriptive.</x:v>
       </x:c>
       <x:c r="B4" s="1"/>
       <x:c r="C4" s="1"/>
@@ -1169,26 +1169,26 @@
       <x:c r="F7" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G7" s="1" t="n">
-        <x:v>40</x:v>
+      <x:c r="G7" s="1" t="str">
+        <x:v>40 + 3 × 10</x:v>
       </x:c>
       <x:c r="H7" s="7" t="n">
-        <x:v>0.979305858261549</x:v>
+        <x:v>0.9793058582615488</x:v>
       </x:c>
       <x:c r="I7" s="7" t="n">
-        <x:v>0.527472527472528</x:v>
+        <x:v>0.5274725274725275</x:v>
       </x:c>
       <x:c r="J7" s="8" t="n">
-        <x:v>0.000291936358002176</x:v>
+        <x:v>0.0002919363580021</x:v>
       </x:c>
       <x:c r="K7" s="7" t="n">
-        <x:v>0.83607019682688</x:v>
+        <x:v>0.8360701968268796</x:v>
       </x:c>
       <x:c r="L7" s="7" t="n">
-        <x:v>0.907139530369058</x:v>
+        <x:v>0.9071395303690584</x:v>
       </x:c>
       <x:c r="M7" s="1" t="str">
-        <x:v>Original retained</x:v>
+        <x:v>W&amp;B: original retained</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26" hidden="0" customHeight="1">
@@ -1498,7 +1498,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G15" s="14" t="str">
-        <x:v>20 + 20</x:v>
+        <x:v>20 + 20 + 3 × 10</x:v>
       </x:c>
       <x:c r="H15" s="11" t="n">
         <x:v>0.8346957124634393</x:v>
@@ -1516,7 +1516,7 @@
         <x:v>0.8443148594326733</x:v>
       </x:c>
       <x:c r="M15" s="14" t="str">
-        <x:v>Original rule retained</x:v>
+        <x:v>W&amp;B: original retained</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" hidden="0" customHeight="1">
@@ -1538,26 +1538,26 @@
       <x:c r="F16" s="15" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G16" s="15" t="n">
-        <x:v>40</x:v>
+      <x:c r="G16" s="15" t="str">
+        <x:v>40 + 3 × 10</x:v>
       </x:c>
       <x:c r="H16" s="10" t="n">
-        <x:v>0.8217582406266473</x:v>
+        <x:v>0.8363565015360088</x:v>
       </x:c>
       <x:c r="I16" s="10" t="n">
-        <x:v>0.8351648351648352</x:v>
+        <x:v>0.8791208791208791</x:v>
       </x:c>
       <x:c r="J16" s="12" t="n">
-        <x:v>0.0593030666510748</x:v>
+        <x:v>0.0590989357719899</x:v>
       </x:c>
       <x:c r="K16" s="10" t="n">
-        <x:v>0.8244050148450794</x:v>
+        <x:v>0.8445732669303685</x:v>
       </x:c>
       <x:c r="L16" s="10" t="n">
-        <x:v>0.8173525522097386</x:v>
+        <x:v>0.8308996735269819</x:v>
       </x:c>
       <x:c r="M16" s="15" t="str">
-        <x:v>Original remains best</x:v>
+        <x:v>W&amp;B: LR3e-5, epoch10</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="26" hidden="0" customHeight="1">
@@ -2578,7 +2578,7 @@
     </x:row>
     <x:row r="43" ht="32" hidden="0" customHeight="1">
       <x:c r="A43" s="1" t="str">
-        <x:v>Precision, TPR, FPR and F0.5 are means when Runs &gt; 1. Historical best selects a period, not the best individual seed.</x:v>
+        <x:v>Runs denotes seeds, not LR trials. Historical multi-run metrics are means. Each W&amp;B method tested 3 rates, one seed.</x:v>
       </x:c>
       <x:c r="B43" s="1"/>
       <x:c r="C43" s="1"/>
@@ -2663,7 +2663,7 @@
     </x:row>
     <x:row r="48" ht="32" hidden="0" customHeight="1">
       <x:c r="A48" s="1" t="str">
-        <x:v>Historical rows preserved. Full-period masked control and annual metrics are in the accompanying comparison report.</x:v>
+        <x:v>Historical rows preserved. Original controls, all attempts and annual metrics are in the W&amp;B fine-tuning report (25 October 2026).</x:v>
       </x:c>
       <x:c r="B48" s="1"/>
       <x:c r="C48" s="1"/>
@@ -2680,7 +2680,7 @@
     </x:row>
     <x:row r="49" ht="24" hidden="0" customHeight="1">
       <x:c r="A49" s="9" t="str">
-        <x:v>Combinations use seed 42 and a reused benchmark. Fusion uses two models; approach 3 adds channels 14, 21, 29.</x:v>
+        <x:v>W&amp;B: seed 42, reused benchmark, calibration-only selection. Extra inputs: 14, 21, 29. Short-no-roll LR1e-5 repeats prior work.</x:v>
       </x:c>
       <x:c r="B49" s="9"/>
       <x:c r="C49" s="9"/>
@@ -2718,9 +2718,9 @@
     <x:row r="70" ht="32" hidden="0" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53a7f9027438424f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7dd9e2cf63842b2"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cae9c66e41e45bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra55c6926b31e4121"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify and report three-method temporal post-processing comparison
</commit_message>
<xml_diff>
--- a/ESA_thesis_results_full_and_historical.xlsx
+++ b/ESA_thesis_results_full_and_historical.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thesis results" sheetId="1" r:id="Rb27b54676ded44e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thesis results" sheetId="1" r:id="Rc86427d121c8460c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2663,7 +2663,7 @@
     </x:row>
     <x:row r="48" ht="32" hidden="0" customHeight="1">
       <x:c r="A48" s="1" t="str">
-        <x:v>Historical rows preserved. Original controls, all attempts and annual metrics are in the W&amp;B fine-tuning report (25 October 2026).</x:v>
+        <x:v>28 October: temporal processing retained all three W&amp;B alarm rules. Scores unchanged. Full comparison is in the temporal-processing report.</x:v>
       </x:c>
       <x:c r="B48" s="1"/>
       <x:c r="C48" s="1"/>
@@ -2718,9 +2718,9 @@
     <x:row r="70" ht="32" hidden="0" customHeight="1"/>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7dd9e2cf63842b2"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4609d6d0c97e4bfa"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra55c6926b31e4121"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8deab1826014105"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>